<commit_message>
Recepción: conteo por cajas en lugar de escaneo de series
Ahora se registra cuántas cajas llegaron y, caja por caja, se elige el
producto (buscador por nombre o código) y cuántas unidades trae. Una caja
puede traer varios productos.

- Barra de avance: cajas registradas vs. cajas que llegaron.
- Corregir cantidades, quitar productos, reabrir o eliminar cajas.
- Vista "Por caja" y "Por producto".
- Excel con el mismo diseño DJI: agrupado por producto, una fila por
  caja (columna "Caja" en lugar de "Series"), subtotales y total
  general; muestra las cajas recibidas junto a la fecha.
- Se conserva el catálogo (productos agregados/editados) sin cambios de
  formato. Si hay una recepción anterior por series, se ofrece pasarla
  a cajas; nunca se borra.
- LEEME y Excel de ejemplo actualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ov8Y76urQAYMH1FrGigoz
</commit_message>
<xml_diff>
--- a/recepcion/EJEMPLO exportacion.xlsx
+++ b/recepcion/EJEMPLO exportacion.xlsx
@@ -11,9 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="50">
-  <si>
-    <t>Fecha:   17/08/2026</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="36">
+  <si>
+    <t>Fecha:   03/10/2026</t>
+  </si>
+  <si>
+    <t>Cajas recibidas:   6</t>
   </si>
   <si>
     <t>Código</t>
@@ -25,149 +28,104 @@
     <t>Cantidad</t>
   </si>
   <si>
-    <t>Series</t>
-  </si>
-  <si>
-    <t>D00058</t>
-  </si>
-  <si>
-    <t>Drone DJI Lito X1 fly more combo RC 2</t>
-  </si>
-  <si>
-    <t>1581FB34C267D003C3WC</t>
-  </si>
-  <si>
-    <t>1581FB34C267C003C2J0</t>
-  </si>
-  <si>
-    <t>1581FB34C266H003B6NM</t>
-  </si>
-  <si>
-    <t>1581FB34C267C003C2LV</t>
-  </si>
-  <si>
-    <t>1581FB34C267C003C2AJ</t>
-  </si>
-  <si>
-    <t>1581FB34C267C003C277</t>
-  </si>
-  <si>
-    <t>TOTAL  D00058  ·  Drone DJI Lito X1 fly more combo RC 2</t>
+    <t>Caja</t>
+  </si>
+  <si>
+    <t>D00017</t>
+  </si>
+  <si>
+    <t>Base estabilizadora DJI Osmo mobile 7</t>
+  </si>
+  <si>
+    <t>Caja 1</t>
+  </si>
+  <si>
+    <t>Caja 5</t>
+  </si>
+  <si>
+    <t>TOTAL  D00017  ·  Base estabilizadora DJI Osmo mobile 7</t>
   </si>
   <si>
     <t>unidades</t>
   </si>
   <si>
+    <t>D00020</t>
+  </si>
+  <si>
+    <t>Estabilizador para camara DJI RS 4 Mini combo</t>
+  </si>
+  <si>
+    <t>Caja 2</t>
+  </si>
+  <si>
+    <t>TOTAL  D00020  ·  Estabilizador para camara DJI RS 4 Mini combo</t>
+  </si>
+  <si>
+    <t>D00062</t>
+  </si>
+  <si>
+    <t>Camara con base DJI Osmo Pocket 4 creator combo</t>
+  </si>
+  <si>
+    <t>Caja 3</t>
+  </si>
+  <si>
+    <t>TOTAL  D00062  ·  Camara con base DJI Osmo Pocket 4 creator combo</t>
+  </si>
+  <si>
+    <t>D00067</t>
+  </si>
+  <si>
+    <t>Grabadora con microfono DJI Mic Mini 2 2TX + 1RX + estuche de carga</t>
+  </si>
+  <si>
+    <t>TOTAL  D00067  ·  Grabadora con microfono DJI Mic Mini 2 2TX + 1RX + estuche de carga</t>
+  </si>
+  <si>
+    <t>D00041</t>
+  </si>
+  <si>
+    <t>Drone DJI Neo 2 fly more combo</t>
+  </si>
+  <si>
+    <t>Caja 4</t>
+  </si>
+  <si>
+    <t>TOTAL  D00041  ·  Drone DJI Neo 2 fly more combo</t>
+  </si>
+  <si>
     <t>D00074</t>
   </si>
   <si>
     <t>Base estabilizadora DJI Osmo Mobile 8P creator combo</t>
   </si>
   <si>
-    <t>AQGVV266131068QL</t>
-  </si>
-  <si>
-    <t>AQGVV26616106EU2</t>
-  </si>
-  <si>
-    <t>AQGVV26615106B1S</t>
-  </si>
-  <si>
-    <t>AQGVV26615106CNG</t>
+    <t>Caja 6</t>
   </si>
   <si>
     <t>TOTAL  D00074  ·  Base estabilizadora DJI Osmo Mobile 8P creator combo</t>
   </si>
   <si>
-    <t>D00062</t>
-  </si>
-  <si>
-    <t>Camara con base DJI Osmo Pocket 4 creator combo</t>
-  </si>
-  <si>
-    <t>ANGVP7A0020GMG</t>
-  </si>
-  <si>
-    <t>ANGVP4M002067E</t>
-  </si>
-  <si>
-    <t>ANGVP730020ES8</t>
-  </si>
-  <si>
-    <t>ANGVP7A0020AWD</t>
-  </si>
-  <si>
-    <t>ANGVP6R0020B2X</t>
-  </si>
-  <si>
-    <t>TOTAL  D00062  ·  Camara con base DJI Osmo Pocket 4 creator combo</t>
-  </si>
-  <si>
-    <t>D00067</t>
-  </si>
-  <si>
-    <t>Grabadora con microfono DJI Mic Mini 2 2TX + 1RX + estuche de carga</t>
-  </si>
-  <si>
-    <t>B3PTP640029T8P</t>
-  </si>
-  <si>
-    <t>B3PTP63002G25F</t>
-  </si>
-  <si>
-    <t>B3PTP630028X2W</t>
-  </si>
-  <si>
-    <t>B3PTP63002PSPT</t>
-  </si>
-  <si>
-    <t>B3PTP640024GG0</t>
-  </si>
-  <si>
-    <t>B3PTP640029GJP</t>
-  </si>
-  <si>
-    <t>B3PTP640024SXR</t>
-  </si>
-  <si>
-    <t>B3PTP5V0022V01</t>
-  </si>
-  <si>
-    <t>TOTAL  D00067  ·  Grabadora con microfono DJI Mic Mini 2 2TX + 1RX + estuche de carga</t>
-  </si>
-  <si>
-    <t>D00041</t>
-  </si>
-  <si>
-    <t>Drone DJI Neo 2 fly more combo</t>
-  </si>
-  <si>
-    <t>1581FA6QC265T01CBY5B</t>
-  </si>
-  <si>
-    <t>1581FA6QC265T01CBZ0Y</t>
-  </si>
-  <si>
-    <t>1581FA6QC265S01CBTHR</t>
-  </si>
-  <si>
-    <t>1581FA6QC265T01CBZFP</t>
-  </si>
-  <si>
-    <t>TOTAL  D00041  ·  Drone DJI Neo 2 fly more combo</t>
+    <t>D00073</t>
+  </si>
+  <si>
+    <t>Base estabilizadora DJI Osmo Mobile 8P advanced tracking combo</t>
+  </si>
+  <si>
+    <t>TOTAL  D00073  ·  Base estabilizadora DJI Osmo Mobile 8P advanced tracking combo</t>
   </si>
   <si>
     <t>TOTAL GENERAL</t>
   </si>
   <si>
-    <t>5 productos</t>
+    <t>7 productos · 6 cajas</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -185,11 +143,6 @@
       <color rgb="FF4A4F59"/>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <color rgb="FF4A4F59"/>
-      <sz val="11"/>
-      <name val="Consolas"/>
     </font>
     <font>
       <b/>
@@ -248,13 +201,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -267,13 +222,10 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -665,7 +617,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:E38"/>
+  <dimension ref="B1:E21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -699,88 +651,86 @@
         <v>0</v>
       </c>
       <c r="C4" s="2"/>
-      <c r="D4" s="3"/>
+      <c r="D4" s="3" t="s">
+        <v>1</v>
+      </c>
       <c r="E4" s="3"/>
     </row>
     <row r="5" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D6" s="6">
-        <v>1</v>
-      </c>
-      <c r="E6" s="8" t="s">
         <v>7</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D7" s="6">
-        <v>1</v>
-      </c>
-      <c r="E7" s="8" t="s">
         <v>8</v>
       </c>
+      <c r="E7" s="7" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" s="6">
-        <v>1</v>
+      <c r="B8" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="8"/>
+      <c r="D8" s="9">
+        <v>15</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" s="6" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D9" s="6">
-        <v>1</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>10</v>
+        <v>3</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" s="6">
-        <v>1</v>
+      <c r="B10" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="8"/>
+      <c r="D10" s="9">
+        <v>3</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>11</v>
@@ -788,394 +738,159 @@
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B11" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="6">
         <v>5</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D11" s="6">
-        <v>1</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>12</v>
+      <c r="E11" s="7" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B12" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="10">
-        <v>6</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>14</v>
+      <c r="B12" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="8"/>
+      <c r="D12" s="9">
+        <v>5</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B13" s="6" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D13" s="6">
-        <v>1</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>17</v>
+        <v>4</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B14" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D14" s="6">
-        <v>1</v>
+      <c r="B14" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="8"/>
+      <c r="D14" s="9">
+        <v>4</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B15" s="6" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="D15" s="6">
-        <v>1</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>19</v>
+        <v>6</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B16" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D16" s="6">
-        <v>1</v>
+      <c r="B16" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="8"/>
+      <c r="D16" s="9">
+        <v>6</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B17" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="10">
-        <v>4</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>14</v>
+      <c r="B17" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="6">
+        <v>10</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B18" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D18" s="6">
-        <v>1</v>
+      <c r="B18" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" s="8"/>
+      <c r="D18" s="9">
+        <v>10</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" s="6" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="D19" s="6">
-        <v>1</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>25</v>
+        <v>6</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B20" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D20" s="6">
-        <v>1</v>
+      <c r="B20" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="8"/>
+      <c r="D20" s="9">
+        <v>6</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B21" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D21" s="6">
-        <v>1</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B22" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D22" s="6">
-        <v>1</v>
-      </c>
-      <c r="E22" s="8" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B23" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="C23" s="9"/>
-      <c r="D23" s="10">
-        <v>5</v>
-      </c>
-      <c r="E23" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B24" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D24" s="6">
-        <v>1</v>
-      </c>
-      <c r="E24" s="8" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B25" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D25" s="6">
-        <v>1</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B26" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D26" s="6">
-        <v>1</v>
-      </c>
-      <c r="E26" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B21" s="10" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B27" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D27" s="6">
-        <v>1</v>
-      </c>
-      <c r="E27" s="8" t="s">
+      <c r="C21" s="10"/>
+      <c r="D21" s="11">
+        <v>49</v>
+      </c>
+      <c r="E21" s="10" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B28" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C28" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D28" s="6">
-        <v>1</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B29" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D29" s="6">
-        <v>1</v>
-      </c>
-      <c r="E29" s="8" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B30" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D30" s="6">
-        <v>1</v>
-      </c>
-      <c r="E30" s="8" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B31" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D31" s="6">
-        <v>1</v>
-      </c>
-      <c r="E31" s="8" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B32" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="C32" s="9"/>
-      <c r="D32" s="10">
-        <v>8</v>
-      </c>
-      <c r="E32" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B33" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C33" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="D33" s="6">
-        <v>1</v>
-      </c>
-      <c r="E33" s="8" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B34" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C34" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="D34" s="6">
-        <v>1</v>
-      </c>
-      <c r="E34" s="8" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B35" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C35" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="D35" s="6">
-        <v>1</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B36" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C36" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="D36" s="6">
-        <v>1</v>
-      </c>
-      <c r="E36" s="8" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="37" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B37" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="C37" s="9"/>
-      <c r="D37" s="10">
-        <v>4</v>
-      </c>
-      <c r="E37" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="38" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B38" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="C38" s="11"/>
-      <c r="D38" s="12">
-        <v>27</v>
-      </c>
-      <c r="E38" s="11" t="s">
-        <v>49</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="11">
     <mergeCell ref="B1:E3"/>
     <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B10:C10"/>
     <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Recepción: Excel con hoja de resumen por producto
- El Excel ahora tiene dos hojas con el mismo diseño DJI:
  1. "Resumen por producto": una fila por producto con el total que
     ingresó y el total general (es la que abre primero).
  2. "Detalle por caja": el cuadro de siempre, con la cantidad de cada
     caja y los subtotales.
- LEEME y Excel de ejemplo actualizados. Versión 20261005a.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ov8Y76urQAYMH1FrGigoz
</commit_message>
<xml_diff>
--- a/recepcion/EJEMPLO exportacion.xlsx
+++ b/recepcion/EJEMPLO exportacion.xlsx
@@ -4,39 +4,82 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Recepción" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Resumen por producto" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Detalle por caja" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="38">
   <si>
     <t>Fecha:   03/10/2026</t>
   </si>
   <si>
+    <t>Cajas: 6</t>
+  </si>
+  <si>
+    <t>Código</t>
+  </si>
+  <si>
+    <t>Descripción</t>
+  </si>
+  <si>
+    <t>Cantidad</t>
+  </si>
+  <si>
+    <t>D00017</t>
+  </si>
+  <si>
+    <t>Base estabilizadora DJI Osmo mobile 7</t>
+  </si>
+  <si>
+    <t>D00020</t>
+  </si>
+  <si>
+    <t>Estabilizador para camara DJI RS 4 Mini combo</t>
+  </si>
+  <si>
+    <t>D00062</t>
+  </si>
+  <si>
+    <t>Camara con base DJI Osmo Pocket 4 creator combo</t>
+  </si>
+  <si>
+    <t>D00067</t>
+  </si>
+  <si>
+    <t>Grabadora con microfono DJI Mic Mini 2 2TX + 1RX + estuche de carga</t>
+  </si>
+  <si>
+    <t>D00040</t>
+  </si>
+  <si>
+    <t>Drone DJI Neo 2</t>
+  </si>
+  <si>
+    <t>D00074</t>
+  </si>
+  <si>
+    <t>Base estabilizadora DJI Osmo Mobile 8P creator combo</t>
+  </si>
+  <si>
+    <t>D00073</t>
+  </si>
+  <si>
+    <t>Base estabilizadora DJI Osmo Mobile 8P advanced tracking combo</t>
+  </si>
+  <si>
+    <t>TOTAL GENERAL   ·   7 productos   ·   6 cajas</t>
+  </si>
+  <si>
     <t>Cajas recibidas:   6</t>
   </si>
   <si>
-    <t>Código</t>
-  </si>
-  <si>
-    <t>Descripción</t>
-  </si>
-  <si>
-    <t>Cantidad</t>
-  </si>
-  <si>
     <t>Caja</t>
   </si>
   <si>
-    <t>D00017</t>
-  </si>
-  <si>
-    <t>Base estabilizadora DJI Osmo mobile 7</t>
-  </si>
-  <si>
     <t>Caja 1</t>
   </si>
   <si>
@@ -49,67 +92,31 @@
     <t>unidades</t>
   </si>
   <si>
-    <t>D00020</t>
-  </si>
-  <si>
-    <t>Estabilizador para camara DJI RS 4 Mini combo</t>
-  </si>
-  <si>
     <t>Caja 2</t>
   </si>
   <si>
     <t>TOTAL  D00020  ·  Estabilizador para camara DJI RS 4 Mini combo</t>
   </si>
   <si>
-    <t>D00062</t>
-  </si>
-  <si>
-    <t>Camara con base DJI Osmo Pocket 4 creator combo</t>
-  </si>
-  <si>
     <t>Caja 3</t>
   </si>
   <si>
     <t>TOTAL  D00062  ·  Camara con base DJI Osmo Pocket 4 creator combo</t>
   </si>
   <si>
-    <t>D00067</t>
-  </si>
-  <si>
-    <t>Grabadora con microfono DJI Mic Mini 2 2TX + 1RX + estuche de carga</t>
-  </si>
-  <si>
     <t>TOTAL  D00067  ·  Grabadora con microfono DJI Mic Mini 2 2TX + 1RX + estuche de carga</t>
   </si>
   <si>
-    <t>D00041</t>
-  </si>
-  <si>
-    <t>Drone DJI Neo 2 fly more combo</t>
-  </si>
-  <si>
     <t>Caja 4</t>
   </si>
   <si>
-    <t>TOTAL  D00041  ·  Drone DJI Neo 2 fly more combo</t>
-  </si>
-  <si>
-    <t>D00074</t>
-  </si>
-  <si>
-    <t>Base estabilizadora DJI Osmo Mobile 8P creator combo</t>
+    <t>TOTAL  D00040  ·  Drone DJI Neo 2</t>
   </si>
   <si>
     <t>Caja 6</t>
   </si>
   <si>
     <t>TOTAL  D00074  ·  Base estabilizadora DJI Osmo Mobile 8P creator combo</t>
-  </si>
-  <si>
-    <t>D00073</t>
-  </si>
-  <si>
-    <t>Base estabilizadora DJI Osmo Mobile 8P advanced tracking combo</t>
   </si>
   <si>
     <t>TOTAL  D00073  ·  Base estabilizadora DJI Osmo Mobile 8P advanced tracking combo</t>
@@ -222,16 +229,16 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -252,6 +259,50 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>171000</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>45000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="904875" cy="495300"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
@@ -617,6 +668,151 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B1:D13"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="3" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="62" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="3" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B5" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B6" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="6">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B7" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B8" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B9" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B10" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B11" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B12" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B13" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="8"/>
+      <c r="D13" s="9">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B1:D3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B13:C13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:E21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -652,7 +848,7 @@
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="3" t="s">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E4" s="3"/>
     </row>
@@ -667,215 +863,215 @@
         <v>4</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>6</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>7</v>
       </c>
       <c r="D6" s="6">
         <v>7</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="7" t="s">
         <v>6</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>7</v>
       </c>
       <c r="D7" s="6">
         <v>8</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="9">
+      <c r="B8" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="10"/>
+      <c r="D8" s="11">
         <v>15</v>
       </c>
-      <c r="E8" s="8" t="s">
-        <v>11</v>
+      <c r="E8" s="10" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" s="6" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D9" s="6">
         <v>3</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="9">
+      <c r="B10" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="10"/>
+      <c r="D10" s="11">
         <v>3</v>
       </c>
-      <c r="E10" s="8" t="s">
-        <v>11</v>
+      <c r="E10" s="10" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B11" s="6" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="D11" s="6">
         <v>5</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B12" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" s="8"/>
-      <c r="D12" s="9">
+      <c r="B12" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="10"/>
+      <c r="D12" s="11">
         <v>5</v>
       </c>
-      <c r="E12" s="8" t="s">
-        <v>11</v>
+      <c r="E12" s="10" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B13" s="6" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="D13" s="6">
         <v>4</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B14" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="8"/>
-      <c r="D14" s="9">
+      <c r="B14" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="10"/>
+      <c r="D14" s="11">
         <v>4</v>
       </c>
-      <c r="E14" s="8" t="s">
-        <v>11</v>
+      <c r="E14" s="10" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B15" s="6" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D15" s="6">
         <v>6</v>
       </c>
       <c r="E15" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B16" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="10"/>
+      <c r="D16" s="11">
+        <v>6</v>
+      </c>
+      <c r="E16" s="10" t="s">
         <v>25</v>
-      </c>
-    </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B16" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="C16" s="8"/>
-      <c r="D16" s="9">
-        <v>6</v>
-      </c>
-      <c r="E16" s="8" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="6" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="D17" s="6">
         <v>10</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B18" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C18" s="8"/>
-      <c r="D18" s="9">
+      <c r="B18" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" s="10"/>
+      <c r="D18" s="11">
         <v>10</v>
       </c>
-      <c r="E18" s="8" t="s">
-        <v>11</v>
+      <c r="E18" s="10" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" s="6" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D19" s="6">
         <v>6</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B20" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C20" s="8"/>
-      <c r="D20" s="9">
+      <c r="B20" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" s="10"/>
+      <c r="D20" s="11">
         <v>6</v>
       </c>
-      <c r="E20" s="8" t="s">
-        <v>11</v>
+      <c r="E20" s="10" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B21" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C21" s="10"/>
-      <c r="D21" s="11">
+      <c r="B21" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" s="8"/>
+      <c r="D21" s="9">
         <v>49</v>
       </c>
-      <c r="E21" s="10" t="s">
-        <v>35</v>
+      <c r="E21" s="8" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>